<commit_message>
feat: ajustar botoes de exportacao/importacao e adicionar modelo de planilha
</commit_message>
<xml_diff>
--- a/modelo_importacao_produtos.xlsx
+++ b/modelo_importacao_produtos.xlsx
@@ -454,16 +454,20 @@
           <t>PRODUTO EXEMPLO</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>19.9</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>19.90</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>22030000</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>10</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>